<commit_message>
fix: 统一目标表写_i + preprocess推导f_table/i_view + 全部案例修正
核心规则变更：
- mapping实体级目标表物理名称统一写 _i（I视图名）
- preprocess从_i推导_f（F表）和_i（I视图）
- rs_input的target改为 {f_table: {schema,table,cn}, i_view: {schema,table,cn}}
- assemble_ts从rs_input取f_table/i_view（不再自己推导）

案例修正：
- 全部12个案例+标准模板：目标表 _f → _i
- RS资产名同步改_i
- 案例002/003用标准模板重建（表头完整）
- _d结尾的明细层表豁免_i检查

check_case.py自检全部通过
</commit_message>
<xml_diff>
--- a/docs/templates/mapping模板.xlsx
+++ b/docs/templates/mapping模板.xlsx
@@ -1195,7 +1195,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>dwl_con_pu_any_f</t>
+          <t>dwl_con_pu_any_i</t>
         </is>
       </c>
       <c r="K2" s="3" t="n"/>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>dwl_con_pu_any_f</t>
+          <t>dwl_con_pu_any_i</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>dwl_con_pu_any_f</t>
+          <t>dwl_con_pu_any_i</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>dwl_con_pu_any_f</t>
+          <t>dwl_con_pu_any_i</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -2280,12 +2280,6 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>赋值</t>
@@ -2326,12 +2320,6 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>赋值</t>
@@ -2372,12 +2360,6 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>赋值</t>
@@ -2418,12 +2400,6 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>赋值</t>

</xml_diff>